<commit_message>
Make tournament configuration and pricing data-driven
</commit_message>
<xml_diff>
--- a/resources/bachelor_player_ratings_shared.xlsx
+++ b/resources/bachelor_player_ratings_shared.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Bet Legs" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Betting Leaderboard" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Player Leaderboard" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Game Rosters" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'App Config'!$A$1:$D$1</definedName>
@@ -231,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -297,6 +298,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2079,13 +2081,73 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" style="19" min="1" max="1"/>
+    <col width="22" customWidth="1" style="19" min="2" max="2"/>
+    <col width="13" customWidth="1" style="19" min="3" max="3"/>
+    <col width="22" customWidth="1" style="19" min="4" max="4"/>
+    <col width="16" customWidth="1" style="19" min="5" max="5"/>
+    <col width="11" customWidth="1" style="19" min="6" max="6"/>
+    <col width="42" customWidth="1" style="19" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>Game ID</t>
+        </is>
+      </c>
+      <c r="B1" s="31" t="inlineStr">
+        <is>
+          <t>Roster Configuration</t>
+        </is>
+      </c>
+      <c r="C1" s="31" t="inlineStr">
+        <is>
+          <t>Team ID</t>
+        </is>
+      </c>
+      <c r="D1" s="31" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="E1" s="31" t="inlineStr">
+        <is>
+          <t>Rotation Share</t>
+        </is>
+      </c>
+      <c r="F1" s="31" t="inlineStr">
+        <is>
+          <t>Active?</t>
+        </is>
+      </c>
+      <c r="G1" s="31" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="19" min="1" max="1"/>
@@ -2317,6 +2379,226 @@
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>STRAIGHT_VIG</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Straight-market overround used for game lines and player props.</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>PARLAY_BASE_VIG</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Base parlay margin applied after joint simulation pricing.</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>REBOUND_LINE_QUANTILE</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Conservative rebound line percentile.</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>ASSIST_LINE_QUANTILE</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Conservative assist line percentile.</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>THREES_LINE_QUANTILE</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Conservative made-three line percentile.</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>COMBO_LINE_QUANTILE</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Conservative combo-prop line percentile.</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>THREE_POINT_RATE_MIN</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Minimum amateur pickup three-point attempt rate.</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>THREE_POINT_RATE_MAX</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Maximum amateur pickup three-point attempt rate.</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>ASSIST_BASE_RATE</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Base chance that a made basket receives an assist.</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>ASSIST_PLAYMAKING_SLOPE</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Assist-rate increase per playmaking rating point.</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>OFFENSIVE_REBOUND_BASE_RATE</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Base chance a miss becomes an offensive rebound.</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>Organizer</t>
         </is>
@@ -9915,7 +10197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="19" min="1" max="1"/>
@@ -10005,6 +10287,36 @@
           <t>Reconciliation</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Game Type</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Team 1 ID</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Team 2 ID</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Bye ID</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Counts Toward Standings?</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Betting Enabled?</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
@@ -10056,6 +10368,26 @@
         <f>IF(NOT($I2),"PENDING",IF(AND($G2=$L2,$H2=$M2),"OK","CHECK PLAYER POINTS"))</f>
         <v/>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>TOURNAMENT</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Team A</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Team B</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Team C</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
@@ -10107,6 +10439,26 @@
         <f>IF(NOT($I3),"PENDING",IF(AND($G3=$L3,$H3=$M3),"OK","CHECK PLAYER POINTS"))</f>
         <v/>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>TOURNAMENT</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Team B</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Team C</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Team A</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
@@ -10157,6 +10509,26 @@
       <c r="N4" s="30">
         <f>IF(NOT($I4),"PENDING",IF(AND($G4=$L4,$H4=$M4),"OK","CHECK PLAYER POINTS"))</f>
         <v/>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>TOURNAMENT</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Team C</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Team A</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Team B</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>